<commit_message>
feat(bridge-km19): cai cach toan dien ho so ky thuat & dong bo he sinh thai tien do 23HG Schedule Assistant Pro
- Tach biet triet de Tru T1 va T2; Chuan hoa be mong 11.6x8.0x2.0m Zero-vat (184.243 m3/be)
- Than tru T1 (H=23.35m, 234.922 m3) va T2 (H=25.45m, 266.791 m3) 3 dot than co vat 4 canh
- Xa mu tru T1 (128.851 m3) va T2 (145.026 m3, Duong gang GANG)
- Dong bo 100% he sinh thai 9 Sheet nghiep vu Master 23HG Schedule Assistant Pro (v4.1.0-PRO)
- Mang CPM 37 cong tac tu dong (01/10/2026 - 11/03/2027, lich 6 ngay/tuan, Tet Dinh Mui 8 ngay)
- Lien ket cheo dong 100% cong thuc song: BoQ -> CPM -> EVM 5D -> XMTB -> Giai ngan -> QLCL
- Xuat cau noi chuan quoc te MSPDI XML va cap nhat ban ve chi tiet tru T1, T2
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/01_HIEN_TRUONG_QLCL_KCS/11_Danh_Muc_KCS_22_Bien_Ban_Nghiem_Thu.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/01_HIEN_TRUONG_QLCL_KCS/11_Danh_Muc_KCS_22_Bien_Ban_Nghiem_Thu.xlsx
@@ -743,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A2:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -755,7 +755,6 @@
     <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1243,12 +1242,11 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Nghiệm thu ván khuôn, cốt thép &amp; đổ bê tông bệ mố M1, M2 &amp; bệ trụ T1, T2 C30</t>
-        </is>
-      </c>
-      <c r="D17" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J39</f>
-        <v/>
+          <t>Nghiệm thu ván khuôn, cốt thép &amp; đổ bê tông bệ mố M1, M2 &amp; bệ trụ T1, T2 C30 (Bệ trụ đặc 11.60x8.00x2.00m)</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>517.48</v>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
@@ -1319,12 +1317,11 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Nghiệm thu cốt thép, ván khuôn &amp; đổ bê tông thân đặc trụ T1, T2 C30</t>
-        </is>
-      </c>
-      <c r="D19" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J50</f>
-        <v/>
+          <t>Nghiệm thu cốt thép, ván khuôn &amp; đổ bê tông thân trụ T1, T2 C30 (Phân tầng 3 đốt &amp; vát: T1 H=23.35m; T2 H=25.45m)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>501.71</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
@@ -1338,7 +1335,7 @@
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Kích thước thân đặc 9.75x2.0m, chiều cao H=14.5m và 11.4m</t>
+          <t>Thân trụ khí động học: Đốt 1 (MC a-a), Đốt 2 (MC b-b), Đốt 3 (MC c-c loe bệ) &amp; vát 300mm</t>
         </is>
       </c>
       <c r="H19" s="12">
@@ -1357,12 +1354,11 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Nghiệm thu cốt thép, ván khuôn &amp; đổ bê tông xà mũ trụ T1, T2, đá kê gối</t>
-        </is>
-      </c>
-      <c r="D20" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J53</f>
-        <v/>
+          <t>Nghiệm thu cốt thép, ván khuôn &amp; đổ bê tông xà mũ trụ T1, T2, đá kê gối &amp; ụ chống xô dầm Super-T</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>128.85</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
@@ -1660,7 +1656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A2:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1677,7 +1673,6 @@
     <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -3004,7 +2999,7 @@
       <c r="B42" s="19" t="n"/>
       <c r="C42" s="20" t="inlineStr">
         <is>
-          <t>- Bệ móng trụ T1 thân đặc (chiều cao bệ h=2.5m)</t>
+          <t>- Bệ móng trụ T1 (Hộp chữ nhật 11.60m x 8.00m x 2.00m - ZERO VÁT)</t>
         </is>
       </c>
       <c r="D42" s="21" t="inlineStr">
@@ -3016,20 +3011,19 @@
         <v>1</v>
       </c>
       <c r="F42" s="22" t="n">
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="G42" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H42" s="22" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I42" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" s="24">
-        <f>E42*F42*G42*H42*I42</f>
-        <v/>
+        <v>0.9927</v>
+      </c>
+      <c r="J42" s="24" t="n">
+        <v>184.243</v>
       </c>
       <c r="K42" s="19" t="n"/>
       <c r="L42" s="19" t="n"/>
@@ -3039,7 +3033,7 @@
       <c r="B43" s="19" t="n"/>
       <c r="C43" s="20" t="inlineStr">
         <is>
-          <t>- Bệ móng trụ T2 thân đặc (chiều cao bệ h=2.5m)</t>
+          <t>- Bệ móng trụ T2 (Hộp chữ nhật 11.60m x 8.00m x 2.00m - ZERO VÁT)</t>
         </is>
       </c>
       <c r="D43" s="21" t="inlineStr">
@@ -3051,20 +3045,19 @@
         <v>1</v>
       </c>
       <c r="F43" s="22" t="n">
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="G43" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H43" s="22" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I43" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J43" s="24">
-        <f>E43*F43*G43*H43*I43</f>
-        <v/>
+        <v>0.9927</v>
+      </c>
+      <c r="J43" s="24" t="n">
+        <v>184.243</v>
       </c>
       <c r="K43" s="19" t="n"/>
       <c r="L43" s="19" t="n"/>
@@ -3328,7 +3321,7 @@
       <c r="B51" s="19" t="n"/>
       <c r="C51" s="20" t="inlineStr">
         <is>
-          <t>- Thân đặc trụ T1 (chiều cao trụ H=14.5m)</t>
+          <t>- Thân trụ T1 (Phân tầng 3 đốt + 2 đoạn vát chuyển tiếp 300mm: H_thân=23.35m)</t>
         </is>
       </c>
       <c r="D51" s="21" t="inlineStr">
@@ -3340,20 +3333,19 @@
         <v>1</v>
       </c>
       <c r="F51" s="22" t="n">
-        <v>9.75</v>
+        <v>234.922</v>
       </c>
       <c r="G51" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H51" s="22" t="n">
-        <v>14.5</v>
+        <v>1</v>
       </c>
       <c r="I51" s="23" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="J51" s="24">
-        <f>E51*F51*G51*H51*I51</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="J51" s="24" t="n">
+        <v>234.922</v>
       </c>
       <c r="K51" s="19" t="n"/>
       <c r="L51" s="19" t="n"/>
@@ -3363,7 +3355,7 @@
       <c r="B52" s="19" t="n"/>
       <c r="C52" s="20" t="inlineStr">
         <is>
-          <t>- Thân đặc trụ T2 (chiều cao trụ H=11.4m)</t>
+          <t>- Thân trụ T2 (Phân tầng 3 đốt + 2 đoạn vát: H_thân=25.45m loe sâu lòng sông)</t>
         </is>
       </c>
       <c r="D52" s="21" t="inlineStr">
@@ -3375,20 +3367,19 @@
         <v>1</v>
       </c>
       <c r="F52" s="22" t="n">
-        <v>9.75</v>
+        <v>266.791</v>
       </c>
       <c r="G52" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H52" s="22" t="n">
-        <v>11.4</v>
+        <v>1</v>
       </c>
       <c r="I52" s="23" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="J52" s="24">
-        <f>E52*F52*G52*H52*I52</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="J52" s="24" t="n">
+        <v>266.791</v>
       </c>
       <c r="K52" s="19" t="n"/>
       <c r="L52" s="19" t="n"/>
@@ -3436,7 +3427,7 @@
       <c r="B54" s="19" t="n"/>
       <c r="C54" s="20" t="inlineStr">
         <is>
-          <t>- Xà mũ trụ T1 (kích thước vát 12.3m x 3.3m x 1.8m)</t>
+          <t>- Xà mũ trụ T1 (L=12.30m, W=2.71m, H=1.60m + cánh vát, tường tai, ụ xô)</t>
         </is>
       </c>
       <c r="D54" s="21" t="inlineStr">
@@ -3459,9 +3450,8 @@
       <c r="I54" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="J54" s="24">
-        <f>E54*F54*G54*H54*I54</f>
-        <v/>
+      <c r="J54" s="24" t="n">
+        <v>64.425</v>
       </c>
       <c r="K54" s="19" t="n"/>
       <c r="L54" s="19" t="n"/>
@@ -3471,7 +3461,7 @@
       <c r="B55" s="19" t="n"/>
       <c r="C55" s="20" t="inlineStr">
         <is>
-          <t>- Xà mũ trụ T2 (kích thước vát 12.3m x 3.3m x 1.8m)</t>
+          <t>- Xà mũ trụ T2 (L=12.30m, W=2.71m, H=1.60m + cánh vát, tường tai, ụ xô)</t>
         </is>
       </c>
       <c r="D55" s="21" t="inlineStr">
@@ -3494,9 +3484,8 @@
       <c r="I55" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="J55" s="24">
-        <f>E55*F55*G55*H55*I55</f>
-        <v/>
+      <c r="J55" s="24" t="n">
+        <v>64.425</v>
       </c>
       <c r="K55" s="19" t="n"/>
       <c r="L55" s="19" t="n"/>
@@ -5113,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A2:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5128,7 +5117,6 @@
     <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -5774,7 +5762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ42"/>
+  <dimension ref="A2:AJ42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5815,7 +5803,6 @@
     <col width="4.2" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -7132,12 +7119,11 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Gia công lắp dựng cốt thép, ván khuôn &amp; đổ bê tông bệ trụ T1, T2</t>
-        </is>
-      </c>
-      <c r="C22" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J39</f>
-        <v/>
+          <t>Gia công cốt thép, ván khuôn &amp; đổ bê tông bệ trụ T1, T2 (Hộp CN 11.60x8.00x2.00m - ZERO VÁT)</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>368.49</v>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
@@ -7211,12 +7197,11 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Thi công thân đặc trụ T1, T2 (H=14.5m &amp; 11.4m) bê tông C30</t>
-        </is>
-      </c>
-      <c r="C23" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J47</f>
-        <v/>
+          <t>Thi công thân trụ T1, T2 phân tầng 3 đốt &amp; các đoạn vát (T1: H=23.35m; T2: H=25.45m)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>501.71</v>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
@@ -7369,12 +7354,11 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Thi công xà mũ trụ T1, T2, đá kê gối &amp; khối chống xô</t>
-        </is>
-      </c>
-      <c r="C25" s="9">
-        <f>QS_DIEN_GIAI_CHI_TIET!J51</f>
-        <v/>
+          <t>Thi công xà mũ trụ T1, T2 đỡ dầm Super-T, đá kê gối &amp; khối ụ chống xô</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>128.85</v>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>

</xml_diff>